<commit_message>
update `UniteD-SRL - run dependency.xlsx`
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run dependency.xlsx
+++ b/results/UniteD-SRL - run dependency.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e3f7d4e32ee84dc4/UniVe/UniteD-SRL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vito\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="11_1EEB9EAE655331664673AAE434FE8CC552D62E15" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DD41D83-4CEC-4D5C-BC79-47AC3B25BF73}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC9A509-0989-4BEC-9348-133E33053764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41895" yWindow="1365" windowWidth="22965" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="10440" windowWidth="38610" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dependency-based" sheetId="1" r:id="rId1"/>
@@ -226,6 +226,13 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -238,13 +245,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -278,10 +278,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -511,32 +507,32 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
       <c r="L1" s="2"/>
-      <c r="M1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="Q1" s="15" t="s">
+      <c r="M1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="Q1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="U1" s="15" t="s">
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="U1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="Y1" s="15" t="s">
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="Y1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
+      <c r="Z1" s="17"/>
+      <c r="AA1" s="17"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
@@ -556,44 +552,44 @@
       <c r="AR1" s="2"/>
     </row>
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="Q2" s="18" t="s">
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="Q2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="U2" s="18" t="s">
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="U2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="Y2" s="18" t="s">
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="Y2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="16"/>
+      <c r="Z2" s="17"/>
+      <c r="AA2" s="17"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
       <c r="AD2" s="2"/>
@@ -613,7 +609,7 @@
       <c r="AR2" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
@@ -701,22 +697,22 @@
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="20" t="b">
+      <c r="B4" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="15" t="b">
         <v>0</v>
       </c>
       <c r="H4" s="1"/>
@@ -738,11 +734,11 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Z4" s="6" t="e">
-        <f t="shared" ref="Z4:Z12" si="1">AVERAGE(J4,N4,R4,V4)</f>
+        <f t="shared" ref="Z4:Z9" si="1">AVERAGE(J4,N4,R4,V4)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AA4" s="7" t="e">
-        <f t="shared" ref="AA4:AA12" si="2">AVERAGE(K4,O4,S4,W4)</f>
+        <f t="shared" ref="AA4:AA9" si="2">AVERAGE(K4,O4,S4,W4)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="AB4" s="6"/>
@@ -765,22 +761,22 @@
     </row>
     <row r="5" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C5" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="20" t="b">
+      <c r="B5" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="15" t="b">
         <v>0</v>
       </c>
       <c r="H5" s="1"/>
@@ -829,22 +825,22 @@
     </row>
     <row r="6" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="20" t="b">
+      <c r="B6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="15" t="b">
         <v>0</v>
       </c>
       <c r="H6" s="1"/>
@@ -893,22 +889,22 @@
     </row>
     <row r="7" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
-      <c r="B7" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="20" t="b">
+      <c r="B7" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="15" t="b">
         <v>0</v>
       </c>
       <c r="H7" s="1"/>
@@ -957,22 +953,22 @@
     </row>
     <row r="8" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="20" t="b">
+      <c r="B8" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="15" t="b">
         <v>1</v>
       </c>
       <c r="H8" s="1"/>
@@ -1021,22 +1017,22 @@
     </row>
     <row r="9" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="20" t="b">
+      <c r="B9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="15" t="b">
         <v>1</v>
       </c>
       <c r="H9" s="1"/>
@@ -1087,73 +1083,73 @@
       <c r="A10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="20" t="b">
+      <c r="B10" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="15" t="b">
         <v>0</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="6">
-        <v>76.61</v>
+        <v>83.5</v>
       </c>
       <c r="J10" s="6">
-        <v>65.27</v>
+        <v>79.5</v>
       </c>
       <c r="K10" s="7">
-        <v>70.48</v>
+        <v>81.45</v>
       </c>
       <c r="L10" s="6"/>
       <c r="M10" s="6">
-        <v>10.09</v>
+        <v>8.8699999999999992</v>
       </c>
       <c r="N10" s="6">
-        <v>3.32</v>
+        <v>5.8</v>
       </c>
       <c r="O10" s="7">
-        <v>5</v>
+        <v>7.01</v>
       </c>
       <c r="Q10" s="6">
-        <v>54.41</v>
+        <v>47.65</v>
       </c>
       <c r="R10" s="6">
-        <v>36.630000000000003</v>
+        <v>48.68</v>
       </c>
       <c r="S10" s="7">
-        <v>43.78</v>
+        <v>48.16</v>
       </c>
       <c r="U10" s="6">
-        <v>28.23</v>
+        <v>31.26</v>
       </c>
       <c r="V10" s="6">
-        <v>20.079999999999998</v>
+        <v>30.92</v>
       </c>
       <c r="W10" s="7">
-        <v>23.47</v>
+        <v>31.09</v>
       </c>
       <c r="Y10" s="6">
         <f>AVERAGE(I10,M10,Q10,U10)</f>
-        <v>42.335000000000001</v>
+        <v>42.82</v>
       </c>
       <c r="Z10" s="6">
         <f>AVERAGE(J10,N10,R10,V10)</f>
-        <v>31.324999999999999</v>
+        <v>41.224999999999994</v>
       </c>
       <c r="AA10" s="7">
         <f>AVERAGE(K10,O10,S10,W10)</f>
-        <v>35.682500000000005</v>
+        <v>41.927500000000002</v>
       </c>
       <c r="AB10" s="6"/>
       <c r="AC10" s="6"/>
@@ -1175,234 +1171,298 @@
     </row>
     <row r="11" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10"/>
-      <c r="B11" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F11" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="20" t="b">
+      <c r="B11" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="15" t="b">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>31.77</v>
+        <v>11.78</v>
       </c>
       <c r="J11">
-        <v>10.66</v>
+        <v>10.95</v>
       </c>
       <c r="K11" s="11">
-        <v>15.96</v>
+        <v>11.35</v>
       </c>
       <c r="M11">
-        <v>55.42</v>
+        <v>59.29</v>
       </c>
       <c r="N11">
-        <v>47.74</v>
+        <v>56.76</v>
       </c>
       <c r="O11" s="11">
-        <v>51.3</v>
+        <v>58</v>
       </c>
       <c r="Q11">
-        <v>34.5</v>
+        <v>10.210000000000001</v>
       </c>
       <c r="R11">
-        <v>7.33</v>
+        <v>8.76</v>
       </c>
       <c r="S11">
-        <v>12.09</v>
+        <v>9.43</v>
       </c>
       <c r="U11">
-        <v>28.77</v>
+        <v>9.6</v>
       </c>
       <c r="V11">
-        <v>4.22</v>
+        <v>7.62</v>
       </c>
       <c r="W11" s="11">
-        <v>7.37</v>
+        <v>8.5</v>
       </c>
       <c r="Y11" s="6">
         <f t="shared" ref="Y11:Y17" si="3">AVERAGE(I11,M11,Q11,U11)</f>
-        <v>37.615000000000002</v>
+        <v>22.72</v>
       </c>
       <c r="Z11" s="6">
         <f t="shared" ref="Z11:Z17" si="4">AVERAGE(J11,N11,R11,V11)</f>
-        <v>17.487500000000001</v>
+        <v>21.022500000000001</v>
       </c>
       <c r="AA11" s="7">
         <f t="shared" ref="AA11:AA17" si="5">AVERAGE(K11,O11,S11,W11)</f>
-        <v>21.68</v>
+        <v>21.82</v>
       </c>
     </row>
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10"/>
-      <c r="B12" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="20" t="b">
+      <c r="B12" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="15" t="b">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>83.32</v>
+        <v>81.319999999999993</v>
       </c>
       <c r="J12">
-        <v>76.83</v>
+        <v>82.15</v>
       </c>
       <c r="K12" s="11">
-        <v>79.94</v>
+        <v>81.73</v>
       </c>
       <c r="M12">
-        <v>59.98</v>
+        <v>61.38</v>
       </c>
       <c r="N12">
-        <v>55.86</v>
+        <v>59.94</v>
       </c>
       <c r="O12" s="11">
-        <v>57.84</v>
+        <v>60.65</v>
       </c>
       <c r="Q12">
-        <v>59.11</v>
+        <v>39.159999999999997</v>
       </c>
       <c r="R12">
-        <v>53.85</v>
+        <v>46.16</v>
       </c>
       <c r="S12" s="11">
-        <v>56.36</v>
+        <v>42.37</v>
       </c>
       <c r="U12">
-        <v>35.46</v>
+        <v>25.57</v>
       </c>
       <c r="V12">
-        <v>30.74</v>
+        <v>27.82</v>
       </c>
       <c r="W12" s="11">
-        <v>32.93</v>
+        <v>26.65</v>
       </c>
       <c r="Y12" s="6">
         <f t="shared" si="3"/>
-        <v>59.467499999999994</v>
+        <v>51.857499999999995</v>
       </c>
       <c r="Z12" s="6">
         <f t="shared" si="4"/>
-        <v>54.32</v>
+        <v>54.017499999999998</v>
       </c>
       <c r="AA12" s="7">
         <f t="shared" si="5"/>
-        <v>56.767499999999998</v>
+        <v>52.85</v>
       </c>
     </row>
     <row r="13" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10"/>
-      <c r="B13" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="K13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="W13" s="11"/>
-      <c r="Y13" s="6" t="e">
+      <c r="B13" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>71.64</v>
+      </c>
+      <c r="J13" s="6">
+        <v>58.48</v>
+      </c>
+      <c r="K13" s="11">
+        <v>64.39</v>
+      </c>
+      <c r="M13" s="6">
+        <v>50.74</v>
+      </c>
+      <c r="N13" s="6">
+        <v>42.33</v>
+      </c>
+      <c r="O13" s="11">
+        <v>46.16</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>64.650000000000006</v>
+      </c>
+      <c r="R13" s="6">
+        <v>51.8</v>
+      </c>
+      <c r="S13" s="11">
+        <v>57.51</v>
+      </c>
+      <c r="U13" s="6">
+        <v>36.61</v>
+      </c>
+      <c r="V13" s="6">
+        <v>27.19</v>
+      </c>
+      <c r="W13" s="11">
+        <v>31.21</v>
+      </c>
+      <c r="Y13" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z13" s="6" t="e">
+        <v>55.91</v>
+      </c>
+      <c r="Z13" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA13" s="7" t="e">
+        <v>44.95</v>
+      </c>
+      <c r="AA13" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>49.817500000000003</v>
       </c>
     </row>
     <row r="14" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10"/>
-      <c r="B14" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="S14" s="11"/>
-      <c r="W14" s="11"/>
-      <c r="Y14" s="6" t="e">
+      <c r="B14" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="6">
+        <v>83.32</v>
+      </c>
+      <c r="J14" s="6">
+        <v>79.87</v>
+      </c>
+      <c r="K14" s="11">
+        <v>81.56</v>
+      </c>
+      <c r="M14" s="6">
+        <v>61.41</v>
+      </c>
+      <c r="N14" s="6">
+        <v>59.63</v>
+      </c>
+      <c r="O14" s="11">
+        <v>60.5</v>
+      </c>
+      <c r="Q14" s="6">
+        <v>50.2</v>
+      </c>
+      <c r="R14" s="6">
+        <v>47.36</v>
+      </c>
+      <c r="S14" s="11">
+        <v>48.74</v>
+      </c>
+      <c r="U14" s="6">
+        <v>68.39</v>
+      </c>
+      <c r="V14" s="6">
+        <v>64.540000000000006</v>
+      </c>
+      <c r="W14" s="11">
+        <v>66.41</v>
+      </c>
+      <c r="Y14" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z14" s="6" t="e">
+        <v>65.83</v>
+      </c>
+      <c r="Z14" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA14" s="7" t="e">
+        <v>62.850000000000009</v>
+      </c>
+      <c r="AA14" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>64.302500000000009</v>
       </c>
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10"/>
-      <c r="B15" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" s="20" t="b">
+      <c r="B15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="15" t="b">
         <v>1</v>
       </c>
       <c r="K15" s="11"/>
@@ -1426,22 +1486,22 @@
       <c r="A16" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="20" t="b">
+      <c r="B16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="b">
         <v>0</v>
       </c>
       <c r="K16" s="11"/>
@@ -1463,22 +1523,22 @@
     </row>
     <row r="17" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
-      <c r="B17" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" s="20" t="b">
+      <c r="B17" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" s="15" t="b">
         <v>1</v>
       </c>
       <c r="H17" s="1"/>
@@ -1514,19 +1574,19 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="1"/>
-      <c r="AF17" s="15"/>
-      <c r="AG17" s="16"/>
-      <c r="AH17" s="16"/>
-      <c r="AI17" s="16"/>
-      <c r="AJ17" s="16"/>
-      <c r="AK17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="17"/>
+      <c r="AH17" s="17"/>
+      <c r="AI17" s="17"/>
+      <c r="AJ17" s="17"/>
+      <c r="AK17" s="17"/>
       <c r="AL17" s="1"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="16"/>
-      <c r="AO17" s="16"/>
-      <c r="AP17" s="16"/>
-      <c r="AQ17" s="16"/>
-      <c r="AR17" s="16"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="17"/>
+      <c r="AO17" s="17"/>
+      <c r="AP17" s="17"/>
+      <c r="AQ17" s="17"/>
+      <c r="AR17" s="17"/>
     </row>
     <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2530,32 +2590,32 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
       <c r="L1" s="2"/>
-      <c r="M1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="Q1" s="15" t="s">
+      <c r="M1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="Q1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="U1" s="15" t="s">
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="U1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="Y1" s="15" t="s">
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="Y1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
+      <c r="Z1" s="17"/>
+      <c r="AA1" s="17"/>
       <c r="AB1" s="2"/>
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
@@ -2575,44 +2635,44 @@
       <c r="AR1" s="2"/>
     </row>
     <row r="2" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="Q2" s="18" t="s">
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="Q2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
-      <c r="U2" s="18" t="s">
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="U2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="Y2" s="18" t="s">
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="Y2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="16"/>
+      <c r="Z2" s="17"/>
+      <c r="AA2" s="17"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
       <c r="AD2" s="2"/>
@@ -2632,7 +2692,7 @@
       <c r="AR2" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
@@ -3307,19 +3367,19 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="1"/>
-      <c r="AF17" s="15"/>
-      <c r="AG17" s="16"/>
-      <c r="AH17" s="16"/>
-      <c r="AI17" s="16"/>
-      <c r="AJ17" s="16"/>
-      <c r="AK17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="17"/>
+      <c r="AH17" s="17"/>
+      <c r="AI17" s="17"/>
+      <c r="AJ17" s="17"/>
+      <c r="AK17" s="17"/>
       <c r="AL17" s="1"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="16"/>
-      <c r="AO17" s="16"/>
-      <c r="AP17" s="16"/>
-      <c r="AQ17" s="16"/>
-      <c r="AR17" s="16"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="17"/>
+      <c r="AO17" s="17"/>
+      <c r="AP17" s="17"/>
+      <c r="AQ17" s="17"/>
+      <c r="AR17" s="17"/>
     </row>
     <row r="18" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4280,6 +4340,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="AF17:AK17"/>
+    <mergeCell ref="AM17:AR17"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="M1:O1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="Q2:S2"/>
@@ -4287,13 +4354,6 @@
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="U2:W2"/>
-    <mergeCell ref="AF17:AK17"/>
-    <mergeCell ref="AM17:AR17"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="U1:W1"/>
-    <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="M1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update `UniteD-SRL - run dependency.xlsx` and `UniteD-SRL - run span.xlsx`
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run dependency.xlsx
+++ b/results/UniteD-SRL - run dependency.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vito\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC9A509-0989-4BEC-9348-133E33053764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14662696-014D-4EAA-8D1F-FD71A14117FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="10440" windowWidth="38610" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7440" yWindow="4500" windowWidth="20460" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dependency-based" sheetId="1" r:id="rId1"/>
@@ -1465,21 +1465,53 @@
       <c r="G15" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="K15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="S15" s="11"/>
-      <c r="W15" s="11"/>
-      <c r="Y15" s="6" t="e">
+      <c r="I15" s="6">
+        <v>84.2</v>
+      </c>
+      <c r="J15" s="6">
+        <v>81.89</v>
+      </c>
+      <c r="K15" s="11">
+        <v>83.03</v>
+      </c>
+      <c r="M15" s="6">
+        <v>63.2</v>
+      </c>
+      <c r="N15" s="6">
+        <v>61.63</v>
+      </c>
+      <c r="O15" s="11">
+        <v>62.4</v>
+      </c>
+      <c r="Q15" s="6">
+        <v>74.319999999999993</v>
+      </c>
+      <c r="R15" s="6">
+        <v>72.95</v>
+      </c>
+      <c r="S15" s="11">
+        <v>73.63</v>
+      </c>
+      <c r="U15" s="6">
+        <v>67.69</v>
+      </c>
+      <c r="V15" s="6">
+        <v>65.25</v>
+      </c>
+      <c r="W15" s="11">
+        <v>66.45</v>
+      </c>
+      <c r="Y15" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z15" s="6" t="e">
+        <v>72.352499999999992</v>
+      </c>
+      <c r="Z15" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA15" s="7" t="e">
+        <v>70.430000000000007</v>
+      </c>
+      <c r="AA15" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>71.377499999999998</v>
       </c>
     </row>
     <row r="16" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4340,6 +4372,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="U2:W2"/>
     <mergeCell ref="AF17:AK17"/>
     <mergeCell ref="AM17:AR17"/>
     <mergeCell ref="I1:K1"/>
@@ -4347,13 +4386,6 @@
     <mergeCell ref="U1:W1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="M1:O1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="U2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>